<commit_message>
Mejoras completas: Seguridad, Logging, Validación, Backups, Tests y Reportes por fechas
- Fase 1: Seguridad con variables de entorno (.env, SECRET_KEY)
- Fase 2: Sistema de logging profesional (logs rotativos, 5 handlers)
- Fase 3: Validación de archivos FAP/FAO y backups automáticos permanentes
- Fase 4: Documentación completa (20+ funciones documentadas)
- Fase 5: Testing automatizado (33 tests unitarios e integración)
- Sistema de reportes por fechas (día específico o período)
- Backups permanentes (limpieza automática desactivada)

Archivos nuevos:
- logger_config.py: Sistema de logging centralizado
- utils.py: Validación y backups
- DOCUMENTACION.md: Documentación de funciones
- test_access_manager.py: Tests unitarios
- test_integration.py: Tests de integración
- TESTS_README.md: Instrucciones de tests
- .env.example: Plantilla de configuración
- .gitignore: Protección de archivos sensibles
</commit_message>
<xml_diff>
--- a/excepciones.xlsx
+++ b/excepciones.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -576,6 +576,36 @@
       </c>
       <c r="F5" s="2" t="n">
         <v>46003</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>16357580</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Roberto Laforcada</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Merca</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Roberto Laforcada (hijo)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>2025-11-22</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>46005</v>
       </c>
     </row>
   </sheetData>

</xml_diff>